<commit_message>
Inclui Outras Deduções da Receita (Lei 194/2022) no cálculo da receita líquida
A coluna 'Outras Deduções da Receita', introduzida pelo STN em 2022 para
registrar a renúncia fiscal da isenção de ICMS sobre combustíveis (LC 194/2022),
passa a ser subtraída em get_valor_liquido junto às deduções de FUNDEB e
Transferências Constitucionais. Para 2019-2021 o valor é zero, portanto a
série histórica anterior permanece inalterada.
</commit_message>
<xml_diff>
--- a/output/demonstrativos_fiscais_MS_2019_2024.xlsx
+++ b/output/demonstrativos_fiscais_MS_2019_2024.xlsx
@@ -731,19 +731,19 @@
         <v>12766.43</v>
       </c>
       <c r="C5" s="6">
-        <v>15132.46</v>
+        <v>15132.11</v>
       </c>
       <c r="D5" s="6">
-        <v>17313.99</v>
+        <v>17309.05</v>
       </c>
       <c r="E5" s="6">
-        <v>20059.51</v>
+        <v>20028.23</v>
       </c>
       <c r="F5" s="6">
-        <v>25405.72</v>
+        <v>21502.98</v>
       </c>
       <c r="G5" s="6">
-        <v>28324.53</v>
+        <v>21899.05</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1">
@@ -757,16 +757,16 @@
         <v>8147.71</v>
       </c>
       <c r="D6" s="7">
-        <v>9750.15</v>
+        <v>9745.75</v>
       </c>
       <c r="E6" s="7">
-        <v>10864.83</v>
+        <v>10836.38</v>
       </c>
       <c r="F6" s="7">
-        <v>15819.61</v>
+        <v>11917.51</v>
       </c>
       <c r="G6" s="7">
-        <v>19784.51</v>
+        <v>13361.22</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1">
@@ -780,16 +780,16 @@
         <v>6116.12</v>
       </c>
       <c r="D7" s="8">
-        <v>7659.26</v>
+        <v>7657.29</v>
       </c>
       <c r="E7" s="8">
-        <v>8498.530000000001</v>
+        <v>8471.25</v>
       </c>
       <c r="F7" s="8">
-        <v>13096.03</v>
+        <v>9194.950000000001</v>
       </c>
       <c r="G7" s="8">
-        <v>16657.68</v>
+        <v>10236.01</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1">
@@ -803,16 +803,16 @@
         <v>320.3</v>
       </c>
       <c r="D8" s="8">
-        <v>346.19</v>
+        <v>345.42</v>
       </c>
       <c r="E8" s="8">
-        <v>373.11</v>
+        <v>372.95</v>
       </c>
       <c r="F8" s="8">
-        <v>428.48</v>
+        <v>428.05</v>
       </c>
       <c r="G8" s="8">
-        <v>456.75</v>
+        <v>455.87</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="18" customHeight="1">
@@ -829,13 +829,13 @@
         <v>5307.34</v>
       </c>
       <c r="E9" s="7">
-        <v>6184.11</v>
+        <v>6184.06</v>
       </c>
       <c r="F9" s="7">
-        <v>6591.16</v>
+        <v>6591.15</v>
       </c>
       <c r="G9" s="7">
-        <v>5643.7</v>
+        <v>5643.69</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="18" customHeight="1">
@@ -869,10 +869,10 @@
         <v>64.11</v>
       </c>
       <c r="C11" s="7">
-        <v>47.62</v>
+        <v>47.28</v>
       </c>
       <c r="D11" s="7">
-        <v>186.97</v>
+        <v>186.77</v>
       </c>
       <c r="E11" s="7">
         <v>671.52</v>
@@ -895,16 +895,16 @@
         <v>1812.24</v>
       </c>
       <c r="D12" s="7">
-        <v>2069.53</v>
+        <v>2069.18</v>
       </c>
       <c r="E12" s="7">
-        <v>2339.06</v>
+        <v>2336.27</v>
       </c>
       <c r="F12" s="7">
-        <v>2357.35</v>
+        <v>2356.74</v>
       </c>
       <c r="G12" s="7">
-        <v>2398.35</v>
+        <v>2396.17</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="18" customHeight="1">
@@ -918,16 +918,16 @@
         <v>15084.83</v>
       </c>
       <c r="D13" s="9">
-        <v>17127.01</v>
+        <v>17122.28</v>
       </c>
       <c r="E13" s="9">
-        <v>19388</v>
+        <v>19356.71</v>
       </c>
       <c r="F13" s="9">
-        <v>24768.13</v>
+        <v>20865.4</v>
       </c>
       <c r="G13" s="9">
-        <v>27826.56</v>
+        <v>21401.08</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1">
@@ -964,7 +964,7 @@
         <v>37</v>
       </c>
       <c r="D15" s="7">
-        <v>109.02</v>
+        <v>109.01</v>
       </c>
       <c r="E15" s="7">
         <v>79.51000000000001</v>
@@ -1033,7 +1033,7 @@
         <v>7.72</v>
       </c>
       <c r="D18" s="8">
-        <v>10.85</v>
+        <v>10.84</v>
       </c>
       <c r="E18" s="8">
         <v>11.85</v>
@@ -1125,16 +1125,16 @@
         <v>15333.31</v>
       </c>
       <c r="D22" s="10">
-        <v>17387.26</v>
+        <v>17382.52</v>
       </c>
       <c r="E22" s="10">
-        <v>19585.25</v>
+        <v>19553.96</v>
       </c>
       <c r="F22" s="10">
-        <v>24975.92</v>
+        <v>21073.19</v>
       </c>
       <c r="G22" s="10">
-        <v>27994.83</v>
+        <v>21569.35</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="18" customHeight="1">
@@ -1424,16 +1424,16 @@
         <v>219.52</v>
       </c>
       <c r="D35" s="11">
-        <v>-549.05</v>
+        <v>-553.79</v>
       </c>
       <c r="E35" s="11">
-        <v>-2797.49</v>
-      </c>
-      <c r="F35" s="10">
-        <v>1444.41</v>
-      </c>
-      <c r="G35" s="10">
-        <v>3807.45</v>
+        <v>-2828.78</v>
+      </c>
+      <c r="F35" s="11">
+        <v>-2458.32</v>
+      </c>
+      <c r="G35" s="11">
+        <v>-2618.03</v>
       </c>
     </row>
   </sheetData>
@@ -1519,19 +1519,19 @@
         <v>3445.08</v>
       </c>
       <c r="C5" s="6">
-        <v>3983.43</v>
+        <v>3983.13</v>
       </c>
       <c r="D5" s="6">
-        <v>4481.02</v>
+        <v>4479.68</v>
       </c>
       <c r="E5" s="6">
-        <v>4732.7</v>
+        <v>4730.23</v>
       </c>
       <c r="F5" s="6">
-        <v>5072.84</v>
+        <v>5071.81</v>
       </c>
       <c r="G5" s="6">
-        <v>5420.94</v>
+        <v>5419.37</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1">
@@ -1542,19 +1542,19 @@
         <v>1144.88</v>
       </c>
       <c r="C6" s="7">
-        <v>1193.27</v>
+        <v>1193.12</v>
       </c>
       <c r="D6" s="7">
-        <v>1358.9</v>
+        <v>1357.57</v>
       </c>
       <c r="E6" s="7">
-        <v>1525.04</v>
+        <v>1523.82</v>
       </c>
       <c r="F6" s="7">
-        <v>1650.71</v>
+        <v>1649.7</v>
       </c>
       <c r="G6" s="7">
-        <v>1789.43</v>
+        <v>1788.22</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="18" customHeight="1">
@@ -1568,16 +1568,16 @@
         <v>358.86</v>
       </c>
       <c r="D7" s="8">
-        <v>435.64</v>
+        <v>435.52</v>
       </c>
       <c r="E7" s="8">
-        <v>516.62</v>
+        <v>516.33</v>
       </c>
       <c r="F7" s="8">
-        <v>591.49</v>
+        <v>591.05</v>
       </c>
       <c r="G7" s="8">
-        <v>663.8099999999999</v>
+        <v>663.52</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1">
@@ -1588,19 +1588,19 @@
         <v>493.52</v>
       </c>
       <c r="C8" s="8">
-        <v>505.54</v>
+        <v>505.39</v>
       </c>
       <c r="D8" s="8">
-        <v>545.85</v>
+        <v>545.09</v>
       </c>
       <c r="E8" s="8">
-        <v>585.98</v>
+        <v>585.36</v>
       </c>
       <c r="F8" s="8">
-        <v>612.77</v>
+        <v>612.39</v>
       </c>
       <c r="G8" s="8">
-        <v>632.79</v>
+        <v>632.39</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="18" customHeight="1">
@@ -1657,7 +1657,7 @@
         <v>8.119999999999999</v>
       </c>
       <c r="C11" s="7">
-        <v>2.24</v>
+        <v>2.22</v>
       </c>
       <c r="D11" s="7">
         <v>13.21</v>
@@ -1680,19 +1680,19 @@
         <v>402.13</v>
       </c>
       <c r="C12" s="7">
-        <v>453.05</v>
+        <v>452.92</v>
       </c>
       <c r="D12" s="7">
-        <v>753.41</v>
+        <v>753.4</v>
       </c>
       <c r="E12" s="7">
-        <v>553.15</v>
+        <v>551.91</v>
       </c>
       <c r="F12" s="7">
-        <v>566.21</v>
+        <v>566.1799999999999</v>
       </c>
       <c r="G12" s="7">
-        <v>713.96</v>
+        <v>713.59</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="18" customHeight="1">
@@ -1703,19 +1703,19 @@
         <v>3436.96</v>
       </c>
       <c r="C13" s="9">
-        <v>3981.19</v>
+        <v>3980.91</v>
       </c>
       <c r="D13" s="9">
-        <v>4467.81</v>
+        <v>4466.47</v>
       </c>
       <c r="E13" s="9">
-        <v>4667.15</v>
+        <v>4664.68</v>
       </c>
       <c r="F13" s="9">
-        <v>4989.38</v>
+        <v>4988.34</v>
       </c>
       <c r="G13" s="9">
-        <v>5363.37</v>
+        <v>5361.8</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1">
@@ -1729,13 +1729,13 @@
         <v>98.34</v>
       </c>
       <c r="D14" s="6">
-        <v>195.11</v>
+        <v>195.1</v>
       </c>
       <c r="E14" s="6">
-        <v>227.11</v>
+        <v>227.09</v>
       </c>
       <c r="F14" s="6">
-        <v>208.93</v>
+        <v>208.92</v>
       </c>
       <c r="G14" s="6">
         <v>202.81</v>
@@ -1752,10 +1752,10 @@
         <v>80.03</v>
       </c>
       <c r="D15" s="7">
-        <v>121.3</v>
+        <v>121.29</v>
       </c>
       <c r="E15" s="7">
-        <v>202.21</v>
+        <v>202.19</v>
       </c>
       <c r="F15" s="7">
         <v>127.59</v>
@@ -1821,10 +1821,10 @@
         <v>10.05</v>
       </c>
       <c r="D18" s="8">
-        <v>11.11</v>
+        <v>11.1</v>
       </c>
       <c r="E18" s="8">
-        <v>13.71</v>
+        <v>13.7</v>
       </c>
       <c r="F18" s="8">
         <v>13.27</v>
@@ -1873,10 +1873,10 @@
         <v>-0</v>
       </c>
       <c r="F20" s="7">
+        <v>0</v>
+      </c>
+      <c r="G20" s="7">
         <v>-0</v>
-      </c>
-      <c r="G20" s="7">
-        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="18" customHeight="1">
@@ -1910,19 +1910,19 @@
         <v>3473.63</v>
       </c>
       <c r="C22" s="10">
-        <v>3999.5</v>
+        <v>3999.22</v>
       </c>
       <c r="D22" s="10">
-        <v>4541.62</v>
+        <v>4540.29</v>
       </c>
       <c r="E22" s="10">
-        <v>4692.05</v>
+        <v>4689.58</v>
       </c>
       <c r="F22" s="10">
-        <v>5070.71</v>
+        <v>5069.67</v>
       </c>
       <c r="G22" s="10">
-        <v>5497.09</v>
+        <v>5495.52</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="18" customHeight="1">
@@ -2209,19 +2209,19 @@
         <v>-359.51</v>
       </c>
       <c r="C35" s="11">
-        <v>-66.19</v>
+        <v>-66.47</v>
       </c>
       <c r="D35" s="11">
-        <v>-110.93</v>
+        <v>-112.26</v>
       </c>
       <c r="E35" s="11">
-        <v>-735.9400000000001</v>
+        <v>-738.4</v>
       </c>
       <c r="F35" s="11">
-        <v>-381.78</v>
+        <v>-382.82</v>
       </c>
       <c r="G35" s="11">
-        <v>-603.29</v>
+        <v>-604.86</v>
       </c>
     </row>
   </sheetData>
@@ -2310,16 +2310,16 @@
         <v>15333.31</v>
       </c>
       <c r="D5" s="6">
-        <v>17387.26</v>
+        <v>17382.52</v>
       </c>
       <c r="E5" s="6">
-        <v>19585.25</v>
+        <v>19553.96</v>
       </c>
       <c r="F5" s="6">
-        <v>24975.92</v>
+        <v>21073.19</v>
       </c>
       <c r="G5" s="6">
-        <v>27994.83</v>
+        <v>21569.35</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1">
@@ -2356,16 +2356,16 @@
         <v>219.52</v>
       </c>
       <c r="D7" s="11">
-        <v>-549.05</v>
+        <v>-553.79</v>
       </c>
       <c r="E7" s="11">
-        <v>-2797.49</v>
-      </c>
-      <c r="F7" s="10">
-        <v>1444.41</v>
-      </c>
-      <c r="G7" s="10">
-        <v>3807.45</v>
+        <v>-2828.78</v>
+      </c>
+      <c r="F7" s="11">
+        <v>-2458.32</v>
+      </c>
+      <c r="G7" s="11">
+        <v>-2618.03</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1">
@@ -2376,10 +2376,10 @@
         <v>87</v>
       </c>
       <c r="C8" s="6">
-        <v>84.63</v>
+        <v>84.28</v>
       </c>
       <c r="D8" s="6">
-        <v>295.99</v>
+        <v>295.78</v>
       </c>
       <c r="E8" s="6">
         <v>751.03</v>
@@ -2399,10 +2399,10 @@
         <v>64.11</v>
       </c>
       <c r="C9" s="7">
-        <v>47.62</v>
+        <v>47.28</v>
       </c>
       <c r="D9" s="7">
-        <v>186.97</v>
+        <v>186.77</v>
       </c>
       <c r="E9" s="7">
         <v>671.52</v>
@@ -2471,7 +2471,7 @@
         <v>7.72</v>
       </c>
       <c r="D12" s="7">
-        <v>10.85</v>
+        <v>10.84</v>
       </c>
       <c r="E12" s="7">
         <v>11.85</v>
@@ -2560,19 +2560,19 @@
         <v>-2194.82</v>
       </c>
       <c r="C16" s="10">
-        <v>52.47</v>
+        <v>52.12</v>
       </c>
       <c r="D16" s="11">
-        <v>-919.0599999999999</v>
+        <v>-924.01</v>
       </c>
       <c r="E16" s="11">
-        <v>-2778.91</v>
-      </c>
-      <c r="F16" s="10">
-        <v>1379.22</v>
-      </c>
-      <c r="G16" s="10">
-        <v>3603.77</v>
+        <v>-2810.2</v>
+      </c>
+      <c r="F16" s="11">
+        <v>-2523.51</v>
+      </c>
+      <c r="G16" s="11">
+        <v>-2821.72</v>
       </c>
     </row>
   </sheetData>
@@ -2658,19 +2658,19 @@
         <v>3473.63</v>
       </c>
       <c r="C5" s="6">
-        <v>3999.5</v>
+        <v>3999.22</v>
       </c>
       <c r="D5" s="6">
-        <v>4541.62</v>
+        <v>4540.29</v>
       </c>
       <c r="E5" s="6">
-        <v>4692.05</v>
+        <v>4689.58</v>
       </c>
       <c r="F5" s="6">
-        <v>5070.71</v>
+        <v>5069.67</v>
       </c>
       <c r="G5" s="6">
-        <v>5497.09</v>
+        <v>5495.52</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="18" customHeight="1">
@@ -2704,19 +2704,19 @@
         <v>-359.51</v>
       </c>
       <c r="C7" s="11">
-        <v>-66.19</v>
+        <v>-66.47</v>
       </c>
       <c r="D7" s="11">
-        <v>-110.93</v>
+        <v>-112.26</v>
       </c>
       <c r="E7" s="11">
-        <v>-735.9400000000001</v>
+        <v>-738.4</v>
       </c>
       <c r="F7" s="11">
-        <v>-381.78</v>
+        <v>-382.82</v>
       </c>
       <c r="G7" s="11">
-        <v>-603.29</v>
+        <v>-604.86</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="18" customHeight="1">
@@ -2727,16 +2727,16 @@
         <v>107.9</v>
       </c>
       <c r="C8" s="6">
-        <v>82.27</v>
+        <v>82.25</v>
       </c>
       <c r="D8" s="6">
-        <v>134.51</v>
+        <v>134.5</v>
       </c>
       <c r="E8" s="6">
-        <v>267.75</v>
+        <v>267.74</v>
       </c>
       <c r="F8" s="6">
-        <v>211.06</v>
+        <v>211.05</v>
       </c>
       <c r="G8" s="6">
         <v>126.66</v>
@@ -2750,7 +2750,7 @@
         <v>8.119999999999999</v>
       </c>
       <c r="C9" s="7">
-        <v>2.24</v>
+        <v>2.22</v>
       </c>
       <c r="D9" s="7">
         <v>13.21</v>
@@ -2822,10 +2822,10 @@
         <v>10.05</v>
       </c>
       <c r="D12" s="7">
-        <v>11.11</v>
+        <v>11.1</v>
       </c>
       <c r="E12" s="7">
-        <v>13.71</v>
+        <v>13.7</v>
       </c>
       <c r="F12" s="7">
         <v>13.27</v>
@@ -2911,19 +2911,19 @@
         <v>-330.88</v>
       </c>
       <c r="C16" s="11">
-        <v>-44.87</v>
+        <v>-45.17</v>
       </c>
       <c r="D16" s="11">
-        <v>-93.26000000000001</v>
+        <v>-94.61</v>
       </c>
       <c r="E16" s="11">
-        <v>-588.42</v>
+        <v>-590.9</v>
       </c>
       <c r="F16" s="11">
-        <v>-324.03</v>
+        <v>-325.07</v>
       </c>
       <c r="G16" s="11">
-        <v>-650.0599999999999</v>
+        <v>-651.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>